<commit_message>
neco? uz jsem to zapomnela
</commit_message>
<xml_diff>
--- a/kodovani/OE_all_kodovani.xlsx
+++ b/kodovani/OE_all_kodovani.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10118"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/klarakrejcarova/Desktop/Sociologie/2024:25/LS/Alkohol/Alkodata/Nepiti-projekt/Nepiti/kodovani/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annamatejkova/Desktop/projekt alkohol/Nepiti/kodovani/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E24B641-0972-F64A-B0B0-EF81258364B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E441F2C6-16A0-5B47-A285-0AF3A02BD673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16360" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16360" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OE all" sheetId="3" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7296" uniqueCount="2222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7307" uniqueCount="2231">
   <si>
     <t>napil jsem se</t>
   </si>
@@ -6716,6 +6716,33 @@
   </si>
   <si>
     <t>Nepociťuji důvod / nenapadlo mě to</t>
+  </si>
+  <si>
+    <t>tělesné zdraví</t>
+  </si>
+  <si>
+    <t>psychická pohoda</t>
+  </si>
+  <si>
+    <t>necítí se opilý/bez kocoviny</t>
+  </si>
+  <si>
+    <t>ušetřím</t>
+  </si>
+  <si>
+    <t>alkohol nechybí/nemá chuť</t>
+  </si>
+  <si>
+    <t>ostatní</t>
+  </si>
+  <si>
+    <t>zdravotní obtíže</t>
+  </si>
+  <si>
+    <t>sociální problémy</t>
+  </si>
+  <si>
+    <t>žádné negativní dopady</t>
   </si>
 </sst>
 </file>
@@ -22833,14 +22860,16 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCF8C145-F05D-5E4D-B0ED-4C8CC48B7836}">
-  <dimension ref="A1:F1072"/>
+  <dimension ref="A1:H1072"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.6640625" customWidth="1"/>
     <col min="2" max="2" width="31.1640625" customWidth="1"/>
+    <col min="6" max="6" width="23.1640625" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>52</v>
       </c>
@@ -22848,7 +22877,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>38</v>
       </c>
@@ -22856,7 +22885,7 @@
         <v>2049</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>40</v>
       </c>
@@ -22864,7 +22893,7 @@
         <v>2098</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>42</v>
       </c>
@@ -22872,11 +22901,11 @@
         <v>2097</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="6"/>
     </row>
-    <row r="6" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>2086</v>
       </c>
@@ -22887,7 +22916,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>2082</v>
       </c>
@@ -22899,7 +22928,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>2085</v>
       </c>
@@ -22910,8 +22939,19 @@
         <f>COUNTIF($C$51:$C$1072,B8)</f>
         <v>143</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F8" t="s">
+        <v>2230</v>
+      </c>
+      <c r="G8">
+        <f>C9</f>
+        <v>452</v>
+      </c>
+      <c r="H8" s="25">
+        <f>(G8/$G$12)*100</f>
+        <v>66.178623718887266</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>2083</v>
       </c>
@@ -22922,8 +22962,19 @@
         <f>COUNTIF($C$51:$C$1072,B9)</f>
         <v>452</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F9" t="s">
+        <v>2229</v>
+      </c>
+      <c r="G9">
+        <f>C22</f>
+        <v>56</v>
+      </c>
+      <c r="H9" s="25">
+        <f t="shared" ref="H9:H11" si="0">(G9/$G$12)*100</f>
+        <v>8.1991215226939964</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>2084</v>
       </c>
@@ -22934,8 +22985,32 @@
         <f>COUNTIF($C$51:$C$1072,B10)</f>
         <v>24</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F10" t="s">
+        <v>2228</v>
+      </c>
+      <c r="G10">
+        <f>C15+C16+C17+C18</f>
+        <v>76</v>
+      </c>
+      <c r="H10" s="25">
+        <f t="shared" si="0"/>
+        <v>11.127379209370424</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F11" t="s">
+        <v>2227</v>
+      </c>
+      <c r="G11">
+        <f>C13+C20+C30+C38+C35+C36</f>
+        <v>99</v>
+      </c>
+      <c r="H11" s="25">
+        <f t="shared" si="0"/>
+        <v>14.494875549048317</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>2081</v>
       </c>
@@ -22944,8 +23019,16 @@
         <f>SUM(C13:C22)</f>
         <v>179</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="G12">
+        <f xml:space="preserve"> SUM(G8:G11)</f>
+        <v>683</v>
+      </c>
+      <c r="H12">
+        <f>(G12/$G$12)*100</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>2066</v>
       </c>
@@ -22953,11 +23036,11 @@
         <v>3</v>
       </c>
       <c r="C13">
-        <f t="shared" ref="C13:C20" si="0">COUNTIF($C$51:$C$1072,B13)</f>
+        <f t="shared" ref="C13:C20" si="1">COUNTIF($C$51:$C$1072,B13)</f>
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>2052</v>
       </c>
@@ -22965,11 +23048,11 @@
         <v>301</v>
       </c>
       <c r="C14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>2053</v>
       </c>
@@ -22977,11 +23060,11 @@
         <v>302</v>
       </c>
       <c r="C15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>2054</v>
       </c>
@@ -22989,7 +23072,7 @@
         <v>303</v>
       </c>
       <c r="C16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
     </row>
@@ -23001,7 +23084,7 @@
         <v>304</v>
       </c>
       <c r="C17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
     </row>
@@ -23013,7 +23096,7 @@
         <v>305</v>
       </c>
       <c r="C18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
     </row>
@@ -23025,7 +23108,7 @@
         <v>306</v>
       </c>
       <c r="C19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
@@ -23037,7 +23120,7 @@
         <v>307</v>
       </c>
       <c r="C20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
     </row>
@@ -23061,7 +23144,7 @@
         <v>311</v>
       </c>
       <c r="C23" s="16">
-        <f t="shared" ref="C23:C28" si="1">COUNTIF($C$51:$C$1072,B23)</f>
+        <f t="shared" ref="C23:C28" si="2">COUNTIF($C$51:$C$1072,B23)</f>
         <v>8</v>
       </c>
     </row>
@@ -23073,7 +23156,7 @@
         <v>312</v>
       </c>
       <c r="C24" s="16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
     </row>
@@ -23085,7 +23168,7 @@
         <v>313</v>
       </c>
       <c r="C25" s="16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>13</v>
       </c>
     </row>
@@ -23097,7 +23180,7 @@
         <v>314</v>
       </c>
       <c r="C26" s="16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>14</v>
       </c>
     </row>
@@ -23109,7 +23192,7 @@
         <v>315</v>
       </c>
       <c r="C27" s="16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
     </row>
@@ -23121,7 +23204,7 @@
         <v>316</v>
       </c>
       <c r="C28" s="16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
     </row>
@@ -23289,8 +23372,8 @@
       </c>
       <c r="B46" s="6"/>
       <c r="C46">
-        <f>C7+C8</f>
-        <v>288</v>
+        <f>C7+C8 +C10</f>
+        <v>312</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -23300,7 +23383,7 @@
       <c r="B47" s="6"/>
       <c r="C47">
         <f>C45-C46</f>
-        <v>734</v>
+        <v>710</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
@@ -34694,6 +34777,7 @@
   </sheetData>
   <autoFilter ref="A50:K1072" xr:uid="{CCF8C145-F05D-5E4D-B0ED-4C8CC48B7836}"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -64638,7 +64722,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="28">
-        <f>(C8/$C$19)*100</f>
+        <f>(C8/$C$14)*100</f>
         <v>79.900744416873451</v>
       </c>
     </row>
@@ -64658,7 +64742,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="28">
-        <f t="shared" ref="E9:E13" si="0">(C9/$C$19)*100</f>
+        <f>(C9/$C$14)*100</f>
         <v>6.4516129032258061</v>
       </c>
     </row>
@@ -64678,7 +64762,7 @@
         <v>8</v>
       </c>
       <c r="E10" s="28">
-        <f t="shared" si="0"/>
+        <f>(C10/$C$14)*100</f>
         <v>8.4367245657568244</v>
       </c>
     </row>
@@ -64698,7 +64782,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="28">
-        <f t="shared" si="0"/>
+        <f>(C11/$C$14)*100</f>
         <v>1.9851116625310175</v>
       </c>
     </row>
@@ -64718,7 +64802,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="28">
-        <f t="shared" si="0"/>
+        <f>(C12/$C$14)*100</f>
         <v>1.240694789081886</v>
       </c>
     </row>
@@ -64738,24 +64822,24 @@
         <v>0</v>
       </c>
       <c r="E13" s="28">
-        <f t="shared" si="0"/>
+        <f>(C13/$C$14)*100</f>
         <v>1.9851116625310175</v>
       </c>
     </row>
-    <row r="19" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B19" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
         <v>2144</v>
       </c>
-      <c r="C19">
+      <c r="C14">
         <f>SUM(C8:C13)</f>
         <v>403</v>
       </c>
-      <c r="D19">
+      <c r="D14">
         <f>SUM(D8:D13)</f>
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="24" spans="15:19" x14ac:dyDescent="0.2">
       <c r="O24" s="1" t="s">
         <v>43</v>
       </c>
@@ -64772,7 +64856,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="25" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="25" spans="15:19" x14ac:dyDescent="0.2">
       <c r="O25">
         <v>21788056</v>
       </c>
@@ -64783,7 +64867,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="26" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="26" spans="15:19" x14ac:dyDescent="0.2">
       <c r="O26">
         <v>21799168</v>
       </c>
@@ -64794,7 +64878,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="27" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="27" spans="15:19" x14ac:dyDescent="0.2">
       <c r="O27">
         <v>21793671</v>
       </c>
@@ -64805,7 +64889,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="28" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="28" spans="15:19" x14ac:dyDescent="0.2">
       <c r="O28">
         <v>21799238</v>
       </c>
@@ -64816,7 +64900,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="29" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="29" spans="15:19" x14ac:dyDescent="0.2">
       <c r="O29">
         <v>21844831</v>
       </c>
@@ -64827,7 +64911,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="30" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="30" spans="15:19" x14ac:dyDescent="0.2">
       <c r="O30">
         <v>21823798</v>
       </c>
@@ -64838,7 +64922,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="31" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="31" spans="15:19" x14ac:dyDescent="0.2">
       <c r="O31">
         <v>21792878</v>
       </c>
@@ -64849,7 +64933,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="32" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="32" spans="15:19" x14ac:dyDescent="0.2">
       <c r="O32">
         <v>21795458</v>
       </c>
@@ -69369,6 +69453,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -69918,18 +70003,15 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>2176</v>
-      </c>
-      <c r="B25">
-        <v>99</v>
+        <v>2177</v>
       </c>
       <c r="C25">
-        <f t="shared" si="2"/>
-        <v>729</v>
+        <f>SUM(C21:C24)</f>
+        <v>293</v>
       </c>
       <c r="D25" s="27">
         <f>(C25/$C$16)*100</f>
-        <v>248.80546075085323</v>
+        <v>100</v>
       </c>
       <c r="F25">
         <v>21782249</v>
@@ -69956,6 +70038,20 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>2176</v>
+      </c>
+      <c r="B27">
+        <v>99</v>
+      </c>
+      <c r="C27">
+        <f>COUNTIF($H$2:$H$1023,B27)</f>
+        <v>729</v>
+      </c>
+      <c r="D27" s="27">
+        <f>(C27/$C$16)*100</f>
+        <v>248.80546075085323</v>
+      </c>
       <c r="F27">
         <v>21782269</v>
       </c>
@@ -81939,6 +82035,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -83873,16 +83970,17 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{895A2234-D396-B741-8CD6-9357BFEECD9A}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:F967"/>
+  <dimension ref="A1:G967"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.5" customWidth="1"/>
     <col min="3" max="3" width="12.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.33203125" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>51</v>
       </c>
@@ -83890,7 +83988,7 @@
         <v>2101</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>38</v>
       </c>
@@ -83898,7 +83996,7 @@
         <v>2049</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>40</v>
       </c>
@@ -83906,17 +84004,17 @@
         <v>2098</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>42</v>
       </c>
       <c r="B4" s="19"/>
     </row>
-    <row r="5" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="6"/>
     </row>
-    <row r="6" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>2086</v>
       </c>
@@ -83927,7 +84025,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>2082</v>
       </c>
@@ -83941,7 +84039,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>2085</v>
       </c>
@@ -83952,8 +84050,19 @@
         <f>COUNTIF($C$45:$C$1068,B8)</f>
         <v>36</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E8" t="s">
+        <v>2222</v>
+      </c>
+      <c r="F8">
+        <f>C19</f>
+        <v>193</v>
+      </c>
+      <c r="G8" s="25">
+        <f>(F8/$F$14)*100</f>
+        <v>31.129032258064516</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>2083</v>
       </c>
@@ -83964,8 +84073,19 @@
         <f>COUNTIF($C$45:$C$1091,B9)</f>
         <v>186</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E9" t="s">
+        <v>2223</v>
+      </c>
+      <c r="F9">
+        <f>C24</f>
+        <v>229</v>
+      </c>
+      <c r="G9" s="25">
+        <f t="shared" ref="G9:G14" si="0">(F9/$F$14)*100</f>
+        <v>36.935483870967744</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>2084</v>
       </c>
@@ -83976,12 +84096,34 @@
         <f>COUNTIF($C$45:$C$1091,B10)</f>
         <v>53</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E10" t="s">
+        <v>2224</v>
+      </c>
+      <c r="F10">
+        <f>C14</f>
+        <v>61</v>
+      </c>
+      <c r="G10" s="25">
+        <f t="shared" si="0"/>
+        <v>9.8387096774193559</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="3"/>
       <c r="B11" s="20"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E11" t="s">
+        <v>2225</v>
+      </c>
+      <c r="F11">
+        <f>C15</f>
+        <v>50</v>
+      </c>
+      <c r="G11" s="25">
+        <f t="shared" si="0"/>
+        <v>8.064516129032258</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>2080</v>
       </c>
@@ -83992,8 +84134,19 @@
         <f>COUNTIF($C$70:$C$1091,B12) + SUM(C13:C17)+C19+C24+C31</f>
         <v>642</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E12" t="s">
+        <v>2226</v>
+      </c>
+      <c r="F12">
+        <f>C13</f>
+        <v>19</v>
+      </c>
+      <c r="G12" s="25">
+        <f t="shared" si="0"/>
+        <v>3.064516129032258</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>2155</v>
       </c>
@@ -84004,8 +84157,19 @@
         <f>COUNTIF($C$70:$C$1091,B13)</f>
         <v>19</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E13" t="s">
+        <v>2227</v>
+      </c>
+      <c r="F13">
+        <f>C31+C17+C16</f>
+        <v>68</v>
+      </c>
+      <c r="G13" s="25">
+        <f t="shared" si="0"/>
+        <v>10.967741935483872</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>2158</v>
       </c>
@@ -84016,8 +84180,16 @@
         <f>COUNTIF($C$70:$C$1091,B14)</f>
         <v>61</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F14">
+        <f>SUM(F8:F13)</f>
+        <v>620</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>2103</v>
       </c>
@@ -84030,7 +84202,7 @@
       </c>
       <c r="E15" s="16"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>2152</v>
       </c>
@@ -94586,5 +94758,6 @@
     <sortCondition ref="B45:B967"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>